<commit_message>
Make volunteer section collapsible on entry form
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Book1.xlsx
+++ b/public/Book1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chroj\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\Secretary Trial Management\cwags_trial_management-master\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5CD5EACA-8D30-4A9A-B75C-8669129195E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{492A58DD-E872-486F-BEE1-5D28A69A040C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{A328956F-6838-49BF-876E-6FE73E16D900}"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{A328956F-6838-49BF-876E-6FE73E16D900}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="73">
   <si>
     <t xml:space="preserve">Trial Recap </t>
   </si>
@@ -223,6 +223,63 @@
   </si>
   <si>
     <t>Submitted by:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THE NUMBERS WILL AUTO FILL </t>
+  </si>
+  <si>
+    <t>from the class tabs.</t>
+  </si>
+  <si>
+    <t>Complete Recap section below.</t>
+  </si>
+  <si>
+    <t>Trial Recap, Class Results Reports, &amp; Judge</t>
+  </si>
+  <si>
+    <t>Evalutation for each judge must be emailed</t>
+  </si>
+  <si>
+    <t>within 14 days following the conclusion of</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the trial to </t>
+  </si>
+  <si>
+    <t>Shirley@c-wags.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment can be made by Paypal (link on </t>
+  </si>
+  <si>
+    <t>Trial Host - Payment web page) or a check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payable to   C-WAGS and mailed to </t>
+  </si>
+  <si>
+    <t>C-WAGS %Shirley Ottmer  3693 Fairview Ave</t>
+  </si>
+  <si>
+    <t>Jackson, MI 49203</t>
+  </si>
+  <si>
+    <t>Mailed checks or money orders on Canadian</t>
+  </si>
+  <si>
+    <t>banks must include an additional $6 for</t>
+  </si>
+  <si>
+    <t>bank fee. Payments can be made through</t>
+  </si>
+  <si>
+    <t>Paypal without the additional expense.</t>
+  </si>
+  <si>
+    <t>Results received past 14 days must include</t>
+  </si>
+  <si>
+    <t>$40 late results fee</t>
   </si>
 </sst>
 </file>
@@ -234,7 +291,7 @@
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -312,6 +369,29 @@
       <name val="Comic Sans MS"/>
       <family val="4"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -556,12 +636,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
@@ -613,23 +694,48 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
@@ -666,9 +772,6 @@
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -705,31 +808,26 @@
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2 2" xfId="2" xr:uid="{125782B8-C3A4-4F53-A1B6-1A1AAE1260D2}"/>
   </cellStyles>
@@ -763,7 +861,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3" descr="page1image52461568">
+        <xdr:cNvPr id="4" name="Picture 3" descr="page1image52461568" hidden="1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12A675B4-0611-4787-8204-DAD3770713C6}"/>
@@ -811,20 +909,20 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>220980</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>397511</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>114299</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2202180</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>443230</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>160018</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="TextBox 4">
+        <xdr:cNvPr id="5" name="TextBox 4" hidden="1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C1BB412-B1CC-4295-B24B-8FC5C7092291}"/>
@@ -834,16 +932,14 @@
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="220980" y="2319020"/>
-          <a:ext cx="1835150" cy="3307080"/>
+        <a:xfrm flipH="1" flipV="1">
+          <a:off x="10875011" y="5378449"/>
+          <a:ext cx="45719" cy="45719"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
+        <a:noFill/>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
             <a:schemeClr val="lt1">
@@ -870,191 +966,6 @@
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Complete Recap section below Also</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Trial Recap, Class Results Reports, &amp; Judge Evaluation for each judge must be emailed within 14 days following the conclusion of the trial to   </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Shirley@c-wags.org</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Payment can be made by Paypal (link on Trial Host  - Payment web page</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>) or  a check Payable to     C-WAGS and mailed to</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>C-WAGS  %Shirley Ottmer   3693 Fairview Ave     Jackson, MI  49203</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Mailed checks or money orders on Canadian banks must include an additional $6 for bank fee. </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Payments can be made through Paypal without the additional expense. </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="accent2">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" u="sng">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Results received past 14 days must include $40 late results fee</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
       </xdr:txBody>
@@ -1076,7 +987,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Picture 9" descr="page1image52461568">
+        <xdr:cNvPr id="10" name="Picture 9" descr="page1image52461568" hidden="1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E65B71B1-CABF-47DF-A60A-6A9931ABB591}"/>
@@ -1124,23 +1035,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>220980</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>195580</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2202180</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>222250</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="TextBox 10">
+        <xdr:cNvPr id="13" name="TextBox 12" hidden="1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CF9FCC5-894A-45E0-8085-CFF1FBBAF0BB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DF1A891-1A60-4925-9C8A-DF3A9915BCB2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1148,15 +1059,13 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="220980" y="2293620"/>
-          <a:ext cx="1847850" cy="3307080"/>
+          <a:off x="8234680" y="3949700"/>
+          <a:ext cx="1245870" cy="971550"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
+        <a:noFill/>
         <a:ln w="9525" cmpd="sng">
           <a:solidFill>
             <a:schemeClr val="lt1">
@@ -1183,189 +1092,72 @@
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Complete Recap section below Also</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
+          <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>466256</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>99371</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>511975</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>145090</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="TextBox 10" hidden="1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2CF9FCC5-894A-45E0-8085-CFF1FBBAF0BB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="220235" flipH="1" flipV="1">
+          <a:off x="13991756" y="5731821"/>
+          <a:ext cx="45719" cy="45719"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Trial Recap, Class Results Reports, &amp; Judge Evaluation for each judge must be emailed within 14 days following the conclusion of the trial to   </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Shirley@c-wags.org</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Payment can be made by Paypal (link on Trial Host  - Payment web page</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>) or  a check Payable to     C-WAGS and mailed to</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>C-WAGS  %Shirley Ottmer   3693 Fairview Ave     Jackson, MI  49203</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Mailed checks or money orders on Canadian banks must include an additional $6 for bank fee. </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Payments can be made through Paypal without the additional expense. </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="accent2">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" u="sng">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Results received past 14 days must include $40 late results fee</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
+          <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
         <a:p>
           <a:endParaRPr lang="en-US" sz="1100"/>
@@ -1389,7 +1181,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 11" descr="page1image52461568">
+        <xdr:cNvPr id="12" name="Picture 11" descr="page1image52461568" hidden="1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{23984E39-3F5D-4C69-8D3F-09FE208DA47A}"/>
@@ -1435,48 +1227,34 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>220980</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>160020</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>576036</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>27215</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2202180</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="912260" cy="718131"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="TextBox 12">
+        <xdr:cNvPr id="2" name="TextBox 1" hidden="1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7DF1A891-1A60-4925-9C8A-DF3A9915BCB2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{19AFF3A6-B2FE-5BE7-1015-79A1493CE06F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="220980" y="2293620"/>
-          <a:ext cx="1847850" cy="3307080"/>
+        <a:xfrm rot="6196167">
+          <a:off x="11760200" y="5010151"/>
+          <a:ext cx="718131" cy="912260"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
+        <a:noFill/>
       </xdr:spPr>
       <xdr:style>
         <a:lnRef idx="0">
@@ -1489,204 +1267,21 @@
           <a:scrgbClr r="0" g="0" b="0"/>
         </a:effectRef>
         <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
+          <a:schemeClr val="tx1"/>
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="0" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Complete Recap section below Also</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Trial Recap, Class Results Reports, &amp; Judge Evaluation for each judge must be emailed within 14 days following the conclusion of the trial to   </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Shirley@c-wags.org</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Payment can be made by Paypal (link on Trial Host  - Payment web page</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>) or  a check Payable to     C-WAGS and mailed to</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>C-WAGS  %Shirley Ottmer   3693 Fairview Ave     Jackson, MI  49203</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Mailed checks or money orders on Canadian banks must include an additional $6 for bank fee. </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100">
-              <a:solidFill>
-                <a:schemeClr val="accent2">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Payments can be made through Paypal without the additional expense. </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="accent2">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" u="sng">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Results received past 14 days must include $40 late results fee</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="+mn-lt"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100"/>
+          <a:endParaRPr lang="en-CA" sz="1100"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2019,25 +1614,25 @@
     <col min="8" max="8" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="49" customFormat="1" ht="28" x14ac:dyDescent="0.35">
-      <c r="A1" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+    <row r="1" spans="1:8" s="28" customFormat="1" ht="28" x14ac:dyDescent="0.35">
+      <c r="A1" s="25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="48" t="s">
+      <c r="E1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="48" t="s">
+      <c r="F1" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="48" t="s">
+      <c r="G1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="48" t="s">
+      <c r="H1" s="27" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2045,7 +1640,7 @@
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="24" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="3" cm="1">
@@ -2281,8 +1876,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="17.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
+      <c r="A9" s="50" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="50"/>
       <c r="C9" s="1"/>
       <c r="D9" s="7" t="s">
         <v>17</v>
@@ -2314,8 +1911,10 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
+      <c r="A10" s="50" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="50"/>
       <c r="C10" s="6"/>
       <c r="D10" s="7" t="s">
         <v>18</v>
@@ -2347,8 +1946,10 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
+      <c r="A11" s="50" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="50"/>
       <c r="C11" s="6"/>
       <c r="D11" s="7" t="s">
         <v>19</v>
@@ -2380,8 +1981,8 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
+      <c r="A12" s="50"/>
+      <c r="B12" s="50"/>
       <c r="C12" s="6"/>
       <c r="D12" s="7" t="s">
         <v>20</v>
@@ -2413,8 +2014,10 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
+      <c r="A13" s="52" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="52"/>
       <c r="C13" s="6"/>
       <c r="D13" s="7" t="s">
         <v>21</v>
@@ -2446,8 +2049,10 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
+      <c r="A14" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="52"/>
       <c r="C14" s="6"/>
       <c r="D14" s="7" t="s">
         <v>22</v>
@@ -2479,8 +2084,10 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
+      <c r="A15" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="52"/>
       <c r="C15" s="6"/>
       <c r="D15" s="7" t="s">
         <v>23</v>
@@ -2512,8 +2119,10 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
+      <c r="A16" s="52" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="52"/>
       <c r="C16" s="6"/>
       <c r="D16" s="7" t="s">
         <v>24</v>
@@ -2545,8 +2154,10 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="6"/>
-      <c r="B17" s="6"/>
+      <c r="A17" s="53" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="52"/>
       <c r="C17" s="6"/>
       <c r="D17" s="7" t="s">
         <v>25</v>
@@ -2578,8 +2189,10 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="6"/>
-      <c r="B18" s="6"/>
+      <c r="A18" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="52"/>
       <c r="C18" s="6"/>
       <c r="D18" s="7" t="s">
         <v>26</v>
@@ -2611,8 +2224,10 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6"/>
+      <c r="A19" s="52" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" s="52"/>
       <c r="C19" s="6"/>
       <c r="D19" s="7" t="s">
         <v>27</v>
@@ -2644,8 +2259,10 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="6"/>
-      <c r="B20" s="6"/>
+      <c r="A20" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="52"/>
       <c r="C20" s="6"/>
       <c r="D20" s="7" t="s">
         <v>28</v>
@@ -2677,8 +2294,10 @@
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="6"/>
-      <c r="B21" s="6"/>
+      <c r="A21" s="52" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="52"/>
       <c r="C21" s="6"/>
       <c r="D21" s="7" t="s">
         <v>29</v>
@@ -2710,8 +2329,10 @@
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="6"/>
-      <c r="B22" s="6"/>
+      <c r="A22" s="52" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="52"/>
       <c r="C22" s="6"/>
       <c r="D22" s="7" t="s">
         <v>30</v>
@@ -2743,8 +2364,8 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6"/>
+      <c r="A23" s="52"/>
+      <c r="B23" s="52"/>
       <c r="C23" s="6"/>
       <c r="D23" s="7" t="s">
         <v>31</v>
@@ -2776,8 +2397,10 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="6"/>
-      <c r="B24" s="6"/>
+      <c r="A24" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="52"/>
       <c r="C24" s="6"/>
       <c r="D24" s="7" t="s">
         <v>32</v>
@@ -2809,8 +2432,10 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A25" s="6"/>
-      <c r="B25" s="6"/>
+      <c r="A25" s="52" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" s="52"/>
       <c r="C25" s="6"/>
       <c r="D25" s="7" t="s">
         <v>33</v>
@@ -2842,8 +2467,10 @@
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A26" s="6"/>
-      <c r="B26" s="6"/>
+      <c r="A26" s="52" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="52"/>
       <c r="C26" s="6"/>
       <c r="D26" s="7" t="s">
         <v>34</v>
@@ -2875,8 +2502,10 @@
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A27" s="6"/>
-      <c r="B27" s="6"/>
+      <c r="A27" s="52" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="52"/>
       <c r="C27" s="6"/>
       <c r="D27" s="7" t="s">
         <v>35</v>
@@ -2908,8 +2537,8 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A28" s="6"/>
-      <c r="B28" s="6"/>
+      <c r="A28" s="52"/>
+      <c r="B28" s="52"/>
       <c r="C28" s="6"/>
       <c r="D28" s="7" t="s">
         <v>36</v>
@@ -2941,8 +2570,10 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="6"/>
-      <c r="B29" s="6"/>
+      <c r="A29" s="52" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="52"/>
       <c r="C29" s="6"/>
       <c r="D29" s="7" t="s">
         <v>37</v>
@@ -2974,8 +2605,10 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6"/>
+      <c r="A30" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" s="52"/>
       <c r="C30" s="6"/>
       <c r="D30" s="7" t="s">
         <v>38</v>
@@ -3006,11 +2639,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="16" x14ac:dyDescent="0.4">
-      <c r="A31" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="6"/>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="50"/>
+      <c r="B31" s="50"/>
       <c r="C31" s="6"/>
       <c r="D31" s="7" t="s">
         <v>40</v>
@@ -3042,8 +2673,8 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A32" s="6"/>
-      <c r="B32" s="6"/>
+      <c r="A32" s="51"/>
+      <c r="B32" s="51"/>
       <c r="C32" s="6"/>
       <c r="D32" s="7" t="s">
         <v>41</v>
@@ -3131,11 +2762,11 @@
         <v>44</v>
       </c>
       <c r="E37" s="19"/>
-      <c r="F37" s="20">
+      <c r="F37" s="30">
         <f ca="1">F36*F34</f>
         <v>0</v>
       </c>
-      <c r="G37" s="21"/>
+      <c r="G37" s="31"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
@@ -3152,55 +2783,55 @@
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
-      <c r="D39" s="22" t="s">
+      <c r="D39" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="E39" s="23"/>
-      <c r="F39" s="24">
+      <c r="E39" s="21"/>
+      <c r="F39" s="22">
         <v>40</v>
       </c>
-      <c r="G39" s="23"/>
-      <c r="H39" s="23"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
-      <c r="D40" s="22"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
+      <c r="D40" s="20"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="23"/>
-      <c r="G41" s="23"/>
-      <c r="H41" s="23"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
+      <c r="D42" s="20"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
-      <c r="D43" s="22"/>
-      <c r="E43" s="23"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="23"/>
-      <c r="H43" s="23"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="21"/>
+      <c r="H43" s="21"/>
     </row>
     <row r="44" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A44" s="8" t="s">
@@ -3208,123 +2839,123 @@
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="23"/>
-      <c r="F44" s="23"/>
-      <c r="G44" s="23"/>
-      <c r="H44" s="23"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="21"/>
+      <c r="H44" s="21"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A45" s="25"/>
-      <c r="B45" s="26"/>
-      <c r="C45" s="26"/>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
-      <c r="H45" s="27"/>
+      <c r="A45" s="32"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="33"/>
+      <c r="G45" s="33"/>
+      <c r="H45" s="34"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A46" s="28"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="29"/>
-      <c r="E46" s="29"/>
-      <c r="F46" s="29"/>
-      <c r="G46" s="29"/>
-      <c r="H46" s="30"/>
+      <c r="A46" s="35"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="36"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
+      <c r="H46" s="37"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A47" s="28"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="29"/>
-      <c r="F47" s="29"/>
-      <c r="G47" s="29"/>
-      <c r="H47" s="30"/>
+      <c r="A47" s="35"/>
+      <c r="B47" s="36"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="36"/>
+      <c r="E47" s="36"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="36"/>
+      <c r="H47" s="37"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A48" s="28"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="29"/>
-      <c r="E48" s="29"/>
-      <c r="F48" s="29"/>
-      <c r="G48" s="29"/>
-      <c r="H48" s="30"/>
+      <c r="A48" s="35"/>
+      <c r="B48" s="36"/>
+      <c r="C48" s="36"/>
+      <c r="D48" s="36"/>
+      <c r="E48" s="36"/>
+      <c r="F48" s="36"/>
+      <c r="G48" s="36"/>
+      <c r="H48" s="37"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A49" s="31"/>
-      <c r="B49" s="32"/>
-      <c r="C49" s="32"/>
-      <c r="D49" s="32"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="32"/>
-      <c r="H49" s="33"/>
+      <c r="A49" s="38"/>
+      <c r="B49" s="39"/>
+      <c r="C49" s="39"/>
+      <c r="D49" s="39"/>
+      <c r="E49" s="39"/>
+      <c r="F49" s="39"/>
+      <c r="G49" s="39"/>
+      <c r="H49" s="40"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
-      <c r="D50" s="22"/>
-      <c r="E50" s="23"/>
-      <c r="F50" s="23"/>
-      <c r="G50" s="23"/>
-      <c r="H50" s="23"/>
+      <c r="D50" s="20"/>
+      <c r="E50" s="21"/>
+      <c r="F50" s="21"/>
+      <c r="G50" s="21"/>
+      <c r="H50" s="21"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A51" s="34" t="s">
+      <c r="A51" s="23" t="s">
         <v>47</v>
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
-      <c r="D51" s="22"/>
-      <c r="E51" s="23"/>
-      <c r="F51" s="23"/>
-      <c r="G51" s="23"/>
-      <c r="H51" s="23"/>
+      <c r="D51" s="20"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="21"/>
+      <c r="G51" s="21"/>
+      <c r="H51" s="21"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A52" s="35"/>
-      <c r="B52" s="36"/>
-      <c r="C52" s="36"/>
-      <c r="D52" s="36"/>
-      <c r="E52" s="36"/>
-      <c r="F52" s="36"/>
-      <c r="G52" s="36"/>
-      <c r="H52" s="37"/>
+      <c r="A52" s="41"/>
+      <c r="B52" s="42"/>
+      <c r="C52" s="42"/>
+      <c r="D52" s="42"/>
+      <c r="E52" s="42"/>
+      <c r="F52" s="42"/>
+      <c r="G52" s="42"/>
+      <c r="H52" s="43"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A53" s="38"/>
-      <c r="B53" s="39"/>
-      <c r="C53" s="39"/>
-      <c r="D53" s="39"/>
-      <c r="E53" s="39"/>
-      <c r="F53" s="39"/>
-      <c r="G53" s="39"/>
-      <c r="H53" s="40"/>
+      <c r="A53" s="44"/>
+      <c r="B53" s="45"/>
+      <c r="C53" s="45"/>
+      <c r="D53" s="45"/>
+      <c r="E53" s="45"/>
+      <c r="F53" s="45"/>
+      <c r="G53" s="45"/>
+      <c r="H53" s="46"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A54" s="41"/>
-      <c r="B54" s="42"/>
-      <c r="C54" s="42"/>
-      <c r="D54" s="42"/>
-      <c r="E54" s="42"/>
-      <c r="F54" s="42"/>
-      <c r="G54" s="42"/>
-      <c r="H54" s="43"/>
+      <c r="A54" s="47"/>
+      <c r="B54" s="48"/>
+      <c r="C54" s="48"/>
+      <c r="D54" s="48"/>
+      <c r="E54" s="48"/>
+      <c r="F54" s="48"/>
+      <c r="G54" s="48"/>
+      <c r="H54" s="49"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
-      <c r="D55" s="22"/>
-      <c r="E55" s="23"/>
-      <c r="F55" s="23"/>
-      <c r="G55" s="23"/>
-      <c r="H55" s="23"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="21"/>
+      <c r="G55" s="21"/>
+      <c r="H55" s="21"/>
     </row>
     <row r="56" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A56" s="8" t="s">
@@ -3332,11 +2963,11 @@
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
-      <c r="D56" s="22"/>
-      <c r="E56" s="23"/>
-      <c r="F56" s="23"/>
-      <c r="G56" s="23"/>
-      <c r="H56" s="23"/>
+      <c r="D56" s="20"/>
+      <c r="E56" s="21"/>
+      <c r="F56" s="21"/>
+      <c r="G56" s="21"/>
+      <c r="H56" s="21"/>
     </row>
     <row r="57" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A57" s="8" t="s">
@@ -3344,195 +2975,195 @@
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
-      <c r="D57" s="22"/>
-      <c r="E57" s="23"/>
-      <c r="F57" s="23"/>
-      <c r="G57" s="23"/>
-      <c r="H57" s="23"/>
+      <c r="D57" s="20"/>
+      <c r="E57" s="21"/>
+      <c r="F57" s="21"/>
+      <c r="G57" s="21"/>
+      <c r="H57" s="21"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A58" s="25"/>
-      <c r="B58" s="26"/>
-      <c r="C58" s="26"/>
-      <c r="D58" s="26"/>
-      <c r="E58" s="26"/>
-      <c r="F58" s="26"/>
-      <c r="G58" s="26"/>
-      <c r="H58" s="27"/>
+      <c r="A58" s="32"/>
+      <c r="B58" s="33"/>
+      <c r="C58" s="33"/>
+      <c r="D58" s="33"/>
+      <c r="E58" s="33"/>
+      <c r="F58" s="33"/>
+      <c r="G58" s="33"/>
+      <c r="H58" s="34"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A59" s="28"/>
-      <c r="B59" s="29"/>
-      <c r="C59" s="29"/>
-      <c r="D59" s="29"/>
-      <c r="E59" s="29"/>
-      <c r="F59" s="29"/>
-      <c r="G59" s="29"/>
-      <c r="H59" s="30"/>
+      <c r="A59" s="35"/>
+      <c r="B59" s="36"/>
+      <c r="C59" s="36"/>
+      <c r="D59" s="36"/>
+      <c r="E59" s="36"/>
+      <c r="F59" s="36"/>
+      <c r="G59" s="36"/>
+      <c r="H59" s="37"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A60" s="28"/>
-      <c r="B60" s="29"/>
-      <c r="C60" s="29"/>
-      <c r="D60" s="29"/>
-      <c r="E60" s="29"/>
-      <c r="F60" s="29"/>
-      <c r="G60" s="29"/>
-      <c r="H60" s="30"/>
+      <c r="A60" s="35"/>
+      <c r="B60" s="36"/>
+      <c r="C60" s="36"/>
+      <c r="D60" s="36"/>
+      <c r="E60" s="36"/>
+      <c r="F60" s="36"/>
+      <c r="G60" s="36"/>
+      <c r="H60" s="37"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A61" s="28"/>
-      <c r="B61" s="29"/>
-      <c r="C61" s="29"/>
-      <c r="D61" s="29"/>
-      <c r="E61" s="29"/>
-      <c r="F61" s="29"/>
-      <c r="G61" s="29"/>
-      <c r="H61" s="30"/>
+      <c r="A61" s="35"/>
+      <c r="B61" s="36"/>
+      <c r="C61" s="36"/>
+      <c r="D61" s="36"/>
+      <c r="E61" s="36"/>
+      <c r="F61" s="36"/>
+      <c r="G61" s="36"/>
+      <c r="H61" s="37"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A62" s="28"/>
-      <c r="B62" s="29"/>
-      <c r="C62" s="29"/>
-      <c r="D62" s="29"/>
-      <c r="E62" s="29"/>
-      <c r="F62" s="29"/>
-      <c r="G62" s="29"/>
-      <c r="H62" s="30"/>
+      <c r="A62" s="35"/>
+      <c r="B62" s="36"/>
+      <c r="C62" s="36"/>
+      <c r="D62" s="36"/>
+      <c r="E62" s="36"/>
+      <c r="F62" s="36"/>
+      <c r="G62" s="36"/>
+      <c r="H62" s="37"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A63" s="28"/>
-      <c r="B63" s="29"/>
-      <c r="C63" s="29"/>
-      <c r="D63" s="29"/>
-      <c r="E63" s="29"/>
-      <c r="F63" s="29"/>
-      <c r="G63" s="29"/>
-      <c r="H63" s="30"/>
+      <c r="A63" s="35"/>
+      <c r="B63" s="36"/>
+      <c r="C63" s="36"/>
+      <c r="D63" s="36"/>
+      <c r="E63" s="36"/>
+      <c r="F63" s="36"/>
+      <c r="G63" s="36"/>
+      <c r="H63" s="37"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A64" s="28"/>
-      <c r="B64" s="29"/>
-      <c r="C64" s="29"/>
-      <c r="D64" s="29"/>
-      <c r="E64" s="29"/>
-      <c r="F64" s="29"/>
-      <c r="G64" s="29"/>
-      <c r="H64" s="30"/>
+      <c r="A64" s="35"/>
+      <c r="B64" s="36"/>
+      <c r="C64" s="36"/>
+      <c r="D64" s="36"/>
+      <c r="E64" s="36"/>
+      <c r="F64" s="36"/>
+      <c r="G64" s="36"/>
+      <c r="H64" s="37"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A65" s="31"/>
-      <c r="B65" s="32"/>
-      <c r="C65" s="32"/>
-      <c r="D65" s="32"/>
-      <c r="E65" s="32"/>
-      <c r="F65" s="32"/>
-      <c r="G65" s="32"/>
-      <c r="H65" s="33"/>
+      <c r="A65" s="38"/>
+      <c r="B65" s="39"/>
+      <c r="C65" s="39"/>
+      <c r="D65" s="39"/>
+      <c r="E65" s="39"/>
+      <c r="F65" s="39"/>
+      <c r="G65" s="39"/>
+      <c r="H65" s="40"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="6"/>
       <c r="B66" s="6"/>
       <c r="C66" s="6"/>
-      <c r="D66" s="22"/>
-      <c r="E66" s="23"/>
-      <c r="F66" s="23"/>
-      <c r="G66" s="23"/>
-      <c r="H66" s="23"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="21"/>
+      <c r="F66" s="21"/>
+      <c r="G66" s="21"/>
+      <c r="H66" s="21"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A67" s="22" t="s">
+      <c r="A67" s="20" t="s">
         <v>50</v>
       </c>
       <c r="B67" s="6"/>
       <c r="C67" s="6"/>
-      <c r="D67" s="22"/>
-      <c r="E67" s="23"/>
-      <c r="F67" s="23"/>
-      <c r="G67" s="23"/>
-      <c r="H67" s="23"/>
+      <c r="D67" s="20"/>
+      <c r="E67" s="21"/>
+      <c r="F67" s="21"/>
+      <c r="G67" s="21"/>
+      <c r="H67" s="21"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A68" s="22" t="s">
+      <c r="A68" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="6"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
-      <c r="G68" s="23"/>
-      <c r="H68" s="23"/>
+      <c r="D68" s="20"/>
+      <c r="E68" s="21"/>
+      <c r="F68" s="21"/>
+      <c r="G68" s="21"/>
+      <c r="H68" s="21"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A69" s="25"/>
-      <c r="B69" s="26"/>
-      <c r="C69" s="26"/>
-      <c r="D69" s="26"/>
-      <c r="E69" s="26"/>
-      <c r="F69" s="26"/>
-      <c r="G69" s="26"/>
-      <c r="H69" s="27"/>
+      <c r="A69" s="32"/>
+      <c r="B69" s="33"/>
+      <c r="C69" s="33"/>
+      <c r="D69" s="33"/>
+      <c r="E69" s="33"/>
+      <c r="F69" s="33"/>
+      <c r="G69" s="33"/>
+      <c r="H69" s="34"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A70" s="28"/>
-      <c r="B70" s="29"/>
-      <c r="C70" s="29"/>
-      <c r="D70" s="29"/>
-      <c r="E70" s="29"/>
-      <c r="F70" s="29"/>
-      <c r="G70" s="29"/>
-      <c r="H70" s="30"/>
+      <c r="A70" s="35"/>
+      <c r="B70" s="36"/>
+      <c r="C70" s="36"/>
+      <c r="D70" s="36"/>
+      <c r="E70" s="36"/>
+      <c r="F70" s="36"/>
+      <c r="G70" s="36"/>
+      <c r="H70" s="37"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A71" s="28"/>
-      <c r="B71" s="29"/>
-      <c r="C71" s="29"/>
-      <c r="D71" s="29"/>
-      <c r="E71" s="29"/>
-      <c r="F71" s="29"/>
-      <c r="G71" s="29"/>
-      <c r="H71" s="30"/>
+      <c r="A71" s="35"/>
+      <c r="B71" s="36"/>
+      <c r="C71" s="36"/>
+      <c r="D71" s="36"/>
+      <c r="E71" s="36"/>
+      <c r="F71" s="36"/>
+      <c r="G71" s="36"/>
+      <c r="H71" s="37"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A72" s="28"/>
-      <c r="B72" s="29"/>
-      <c r="C72" s="29"/>
-      <c r="D72" s="29"/>
-      <c r="E72" s="29"/>
-      <c r="F72" s="29"/>
-      <c r="G72" s="29"/>
-      <c r="H72" s="30"/>
+      <c r="A72" s="35"/>
+      <c r="B72" s="36"/>
+      <c r="C72" s="36"/>
+      <c r="D72" s="36"/>
+      <c r="E72" s="36"/>
+      <c r="F72" s="36"/>
+      <c r="G72" s="36"/>
+      <c r="H72" s="37"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A73" s="28"/>
-      <c r="B73" s="29"/>
-      <c r="C73" s="29"/>
-      <c r="D73" s="29"/>
-      <c r="E73" s="29"/>
-      <c r="F73" s="29"/>
-      <c r="G73" s="29"/>
-      <c r="H73" s="30"/>
+      <c r="A73" s="35"/>
+      <c r="B73" s="36"/>
+      <c r="C73" s="36"/>
+      <c r="D73" s="36"/>
+      <c r="E73" s="36"/>
+      <c r="F73" s="36"/>
+      <c r="G73" s="36"/>
+      <c r="H73" s="37"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A74" s="31"/>
-      <c r="B74" s="32"/>
-      <c r="C74" s="32"/>
-      <c r="D74" s="32"/>
-      <c r="E74" s="32"/>
-      <c r="F74" s="32"/>
-      <c r="G74" s="32"/>
-      <c r="H74" s="33"/>
+      <c r="A74" s="38"/>
+      <c r="B74" s="39"/>
+      <c r="C74" s="39"/>
+      <c r="D74" s="39"/>
+      <c r="E74" s="39"/>
+      <c r="F74" s="39"/>
+      <c r="G74" s="39"/>
+      <c r="H74" s="40"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="6"/>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
-      <c r="D75" s="22"/>
-      <c r="E75" s="23"/>
-      <c r="F75" s="23"/>
-      <c r="G75" s="23"/>
-      <c r="H75" s="23"/>
+      <c r="D75" s="20"/>
+      <c r="E75" s="21"/>
+      <c r="F75" s="21"/>
+      <c r="G75" s="21"/>
+      <c r="H75" s="21"/>
     </row>
     <row r="76" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A76" s="8" t="s">
@@ -3540,91 +3171,91 @@
       </c>
       <c r="B76" s="6"/>
       <c r="C76" s="6"/>
-      <c r="D76" s="22"/>
-      <c r="E76" s="23"/>
-      <c r="F76" s="23"/>
-      <c r="G76" s="23"/>
-      <c r="H76" s="23"/>
+      <c r="D76" s="20"/>
+      <c r="E76" s="21"/>
+      <c r="F76" s="21"/>
+      <c r="G76" s="21"/>
+      <c r="H76" s="21"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A77" s="25"/>
-      <c r="B77" s="26"/>
-      <c r="C77" s="26"/>
-      <c r="D77" s="26"/>
-      <c r="E77" s="26"/>
-      <c r="F77" s="26"/>
-      <c r="G77" s="26"/>
-      <c r="H77" s="27"/>
+      <c r="A77" s="32"/>
+      <c r="B77" s="33"/>
+      <c r="C77" s="33"/>
+      <c r="D77" s="33"/>
+      <c r="E77" s="33"/>
+      <c r="F77" s="33"/>
+      <c r="G77" s="33"/>
+      <c r="H77" s="34"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A78" s="28"/>
-      <c r="B78" s="29"/>
-      <c r="C78" s="29"/>
-      <c r="D78" s="29"/>
-      <c r="E78" s="29"/>
-      <c r="F78" s="29"/>
-      <c r="G78" s="29"/>
-      <c r="H78" s="30"/>
+      <c r="A78" s="35"/>
+      <c r="B78" s="36"/>
+      <c r="C78" s="36"/>
+      <c r="D78" s="36"/>
+      <c r="E78" s="36"/>
+      <c r="F78" s="36"/>
+      <c r="G78" s="36"/>
+      <c r="H78" s="37"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A79" s="28"/>
-      <c r="B79" s="29"/>
-      <c r="C79" s="29"/>
-      <c r="D79" s="29"/>
-      <c r="E79" s="29"/>
-      <c r="F79" s="29"/>
-      <c r="G79" s="29"/>
-      <c r="H79" s="30"/>
+      <c r="A79" s="35"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="36"/>
+      <c r="D79" s="36"/>
+      <c r="E79" s="36"/>
+      <c r="F79" s="36"/>
+      <c r="G79" s="36"/>
+      <c r="H79" s="37"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A80" s="28"/>
-      <c r="B80" s="29"/>
-      <c r="C80" s="29"/>
-      <c r="D80" s="29"/>
-      <c r="E80" s="29"/>
-      <c r="F80" s="29"/>
-      <c r="G80" s="29"/>
-      <c r="H80" s="30"/>
+      <c r="A80" s="35"/>
+      <c r="B80" s="36"/>
+      <c r="C80" s="36"/>
+      <c r="D80" s="36"/>
+      <c r="E80" s="36"/>
+      <c r="F80" s="36"/>
+      <c r="G80" s="36"/>
+      <c r="H80" s="37"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A81" s="28"/>
-      <c r="B81" s="29"/>
-      <c r="C81" s="29"/>
-      <c r="D81" s="29"/>
-      <c r="E81" s="29"/>
-      <c r="F81" s="29"/>
-      <c r="G81" s="29"/>
-      <c r="H81" s="30"/>
+      <c r="A81" s="35"/>
+      <c r="B81" s="36"/>
+      <c r="C81" s="36"/>
+      <c r="D81" s="36"/>
+      <c r="E81" s="36"/>
+      <c r="F81" s="36"/>
+      <c r="G81" s="36"/>
+      <c r="H81" s="37"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A82" s="28"/>
-      <c r="B82" s="29"/>
-      <c r="C82" s="29"/>
-      <c r="D82" s="29"/>
-      <c r="E82" s="29"/>
-      <c r="F82" s="29"/>
-      <c r="G82" s="29"/>
-      <c r="H82" s="30"/>
+      <c r="A82" s="35"/>
+      <c r="B82" s="36"/>
+      <c r="C82" s="36"/>
+      <c r="D82" s="36"/>
+      <c r="E82" s="36"/>
+      <c r="F82" s="36"/>
+      <c r="G82" s="36"/>
+      <c r="H82" s="37"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A83" s="31"/>
-      <c r="B83" s="32"/>
-      <c r="C83" s="32"/>
-      <c r="D83" s="32"/>
-      <c r="E83" s="32"/>
-      <c r="F83" s="32"/>
-      <c r="G83" s="32"/>
-      <c r="H83" s="33"/>
+      <c r="A83" s="38"/>
+      <c r="B83" s="39"/>
+      <c r="C83" s="39"/>
+      <c r="D83" s="39"/>
+      <c r="E83" s="39"/>
+      <c r="F83" s="39"/>
+      <c r="G83" s="39"/>
+      <c r="H83" s="40"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="6"/>
       <c r="B84" s="6"/>
       <c r="C84" s="6"/>
-      <c r="D84" s="22"/>
-      <c r="E84" s="23"/>
-      <c r="F84" s="23"/>
-      <c r="G84" s="23"/>
-      <c r="H84" s="23"/>
+      <c r="D84" s="20"/>
+      <c r="E84" s="21"/>
+      <c r="F84" s="21"/>
+      <c r="G84" s="21"/>
+      <c r="H84" s="21"/>
     </row>
     <row r="85" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A85" s="8" t="s">
@@ -3632,44 +3263,68 @@
       </c>
       <c r="B85" s="6"/>
       <c r="C85" s="6"/>
-      <c r="D85" s="22"/>
-      <c r="E85" s="23"/>
-      <c r="F85" s="23"/>
-      <c r="G85" s="23"/>
-      <c r="H85" s="23"/>
+      <c r="D85" s="20"/>
+      <c r="E85" s="21"/>
+      <c r="F85" s="21"/>
+      <c r="G85" s="21"/>
+      <c r="H85" s="21"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A86" s="44"/>
-      <c r="B86" s="44"/>
+      <c r="A86" s="29"/>
+      <c r="B86" s="29"/>
       <c r="C86" s="6"/>
-      <c r="D86" s="22"/>
-      <c r="E86" s="23"/>
-      <c r="F86" s="23"/>
-      <c r="G86" s="23"/>
-      <c r="H86" s="23"/>
+      <c r="D86" s="20"/>
+      <c r="E86" s="21"/>
+      <c r="F86" s="21"/>
+      <c r="G86" s="21"/>
+      <c r="H86" s="21"/>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A87" s="44"/>
-      <c r="B87" s="44"/>
+      <c r="A87" s="29"/>
+      <c r="B87" s="29"/>
       <c r="C87" s="6"/>
-      <c r="D87" s="22"/>
-      <c r="E87" s="23"/>
-      <c r="F87" s="23"/>
-      <c r="G87" s="23"/>
-      <c r="H87" s="23"/>
+      <c r="D87" s="20"/>
+      <c r="E87" s="21"/>
+      <c r="F87" s="21"/>
+      <c r="G87" s="21"/>
+      <c r="H87" s="21"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A88" s="44"/>
-      <c r="B88" s="44"/>
+      <c r="A88" s="29"/>
+      <c r="B88" s="29"/>
       <c r="C88" s="6"/>
-      <c r="D88" s="22"/>
-      <c r="E88" s="23"/>
-      <c r="F88" s="23"/>
-      <c r="G88" s="23"/>
-      <c r="H88" s="23"/>
+      <c r="D88" s="20"/>
+      <c r="E88" s="21"/>
+      <c r="F88" s="21"/>
+      <c r="G88" s="21"/>
+      <c r="H88" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="31">
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A86:B88"/>
     <mergeCell ref="F37:G37"/>
     <mergeCell ref="A45:H49"/>
@@ -3678,7 +3333,10 @@
     <mergeCell ref="A69:H74"/>
     <mergeCell ref="A77:H83"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A17" r:id="rId1" xr:uid="{56DCD14B-8B4E-4B5E-827B-70E9934D4E69}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>